<commit_message>
4. Chapter Distance MAp Registration DONE (FINALLY first version)
</commit_message>
<xml_diff>
--- a/data/distance-maps/iilabs3d/distance-maps_iilabs3d_analysis_range.xlsx
+++ b/data/distance-maps/iilabs3d/distance-maps_iilabs3d_analysis_range.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30121"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30117"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{556722B6-D267-48FC-87AE-FB335625EBFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B17F5C55-1B4A-401A-9D18-1CAFD841FB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dmap p2p (M0) range" sheetId="11" r:id="rId1"/>

</xml_diff>